<commit_message>
Update AFW team guides, Streamlit app, and dashboard data
</commit_message>
<xml_diff>
--- a/workspace/templates/AFW_Eval_Test_Cases_Template.xlsx
+++ b/workspace/templates/AFW_Eval_Test_Cases_Template.xlsx
@@ -18,16 +18,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +35,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -46,21 +43,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -426,16 +414,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>topic</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>detail</t>
         </is>
@@ -461,89 +449,101 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Keep test cases on sheet named: test_cases (or 120_test_cases for legacy).</t>
+          <t>Must be exactly: test_cases (or legacy 120_test_cases). No other sheet names.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>persona_id</t>
+          <t>Strict template</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Unique ID per row (e.g. F001). Required.</t>
+          <t>Column names and order must match this template exactly. Custom uploads that deviate will be rejected by the agent.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>simulated_user_message</t>
+          <t>persona_id</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Opening user message before Q1. Required.</t>
+          <t>Unique ID per row (e.g. F001). Required.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>i–viii. user input message</t>
+          <t>simulated_user_message</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Eight screening answers posted in order. Leave blank if persona stops early.</t>
+          <t>Opening user message before Q1. Required.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>i–viii. manual label</t>
+          <t>i–viii. user input message</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Gold labels per question for scoring only (eligible, ineligible, manual_review, insufficient_information or 1/0/2/3).</t>
+          <t>Eight screening answers posted in order. Leave blank if persona stops early.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ix. final eligibility outcome</t>
+          <t>i–viii. manual label</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Gold final 4-class outcome. Required for accuracy scoring.</t>
+          <t>Gold labels per question for scoring only (eligible, ineligible, manual_review, insufficient_information or 1/0/2/3).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>engineered_for</t>
+          <t>ix. final eligibility outcome</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Optional metadata for analysis — never sent to the chatbot.</t>
+          <t>Gold final 4-class outcome. Required for accuracy scoring.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>engineered_for</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Optional metadata for analysis — never sent to the chatbot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>API endpoints</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>OpenAI host: https://angel-flight-chatbot-app.azurewebsites.net/api/chat | Claude host: https://angel-flight-chatbot-claude.azurewebsites.net/api/chat</t>
         </is>
@@ -564,112 +564,112 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>persona_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>engineered_for</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>simulated_user_message</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>i. user input message</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>i. manual label</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>ii. user input message</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>ii. manual label</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>iii. user input message</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>iii. manual label</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>iv. user input message</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>iv. manual label</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>v. user input message</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>v. manual label</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>vi. user input message</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>vi. manual label</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>vii. user input message</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>vii. manual label</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>viii. user input message</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>viii. manual label</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>ix. final eligibility outcome</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>ix. manual label</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>labeler notes</t>
         </is>

</xml_diff>